<commit_message>
eliminei as linhas ocultas, pois estavam gerando itens desnecessários na ficha de EPIs
</commit_message>
<xml_diff>
--- a/equipamentos.xlsx
+++ b/equipamentos.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Leonardo\Documents\LEONARDO\Gerador-de-fichas-de-EPI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Leonardo GAP\Documents\Gerador-de-fichas-de-EPI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3977AD7-2559-425B-88EE-6AE6013085F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C745BF9-17DD-4398-94A9-5229AA91578B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="3" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -216,7 +216,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1"/>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
@@ -229,7 +229,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="8">
     <cellStyle name="Data" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -699,7 +698,9 @@
       <c r="A14" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B14" s="4"/>
+      <c r="B14" s="4">
+        <v>27971</v>
+      </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
@@ -753,7 +754,9 @@
       <c r="A22" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B22" s="4"/>
+      <c r="B22" s="4">
+        <v>39416</v>
+      </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
@@ -767,28 +770,36 @@
       <c r="A24" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B24" s="4"/>
+      <c r="B24" s="4">
+        <v>19072</v>
+      </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B25" s="4"/>
+      <c r="B25" s="4">
+        <v>40288</v>
+      </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B26" s="4"/>
+      <c r="B26" s="4">
+        <v>40288</v>
+      </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B27" s="4"/>
+      <c r="B27" s="4">
+        <v>10258</v>
+      </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A28" s="6" t="s">
+      <c r="A28" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B28" s="4">
@@ -845,6 +856,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101005C25850FC8DE9B4F9FFF86415CB592F7" ma:contentTypeVersion="15" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="3274bb2186977023e992677584115b66">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3a415345-6a39-4751-b960-4fc8f12baef7" xmlns:ns3="74ad866f-79dd-4f7a-ba3c-81e3e663768c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="cdea2f78ed261d5e205b95494e30ab76" ns2:_="" ns3:_="">
     <xsd:import namespace="3a415345-6a39-4751-b960-4fc8f12baef7"/>
@@ -1079,15 +1099,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A35E0B0E-C51E-4A81-A983-6DDB77691070}">
   <ds:schemaRefs>
@@ -1100,6 +1111,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EEC5ED25-E853-4E69-964F-CC2E03744A0E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{313301D7-37BC-40D9-8AB2-B5498014B342}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1116,12 +1135,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EEC5ED25-E853-4E69-964F-CC2E03744A0E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>